<commit_message>
feat: add IO list validation sheet
</commit_message>
<xml_diff>
--- a/output/io_list_report.xlsx
+++ b/output/io_list_report.xlsx
@@ -10,10 +10,12 @@
     <sheet name="SUMMARY" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="INPUT" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="OUTPUT" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="ERROR" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'INPUT'!$A$1:$H$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'INPUT'!$A$1:$H$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'OUTPUT'!$A$1:$H$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'ERROR'!$A$1:$E$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -453,7 +455,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
@@ -463,7 +465,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
@@ -483,7 +485,17 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>21</v>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Warnings</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -497,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -506,7 +518,7 @@
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="25" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="65" customWidth="1" min="7" max="7"/>
     <col width="31" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -1270,8 +1282,122 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>INPUT</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>X97</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>151</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>99TestWarnging.csv</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Stores current value in D2000</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>99TestWarnging.csv:161</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>INPUT</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>X98</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>152</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>99TestWarnging.csv</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Count enable command:OFF</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>99TestWarnging.csv:145</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>INPUT</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>X99</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>153</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>99TestWarnging.csv</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Count enable command:ON</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>99TestWarnging.csv:129</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H20"/>
+  <autoFilter ref="A1:H23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1417,4 +1543,161 @@
   <autoFilter ref="A1:H3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="65" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Level</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Message</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>MULTIPLE_USED_FILES</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>X57</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Device is used in multiple files.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>04Lcnt1.csv,08LcPre.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>MULTIPLE_LOGIC_NOTES</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>X57</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Device has multiple logic notes.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Stores latch cnt val 1 in D2002,Stores latch cnt value in D2002</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>MULTIPLE_LOGIC_NOTES</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>X5C</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Device has multiple logic notes.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Coinc sgnl 1 reset cmd:OFF,Coinc sgnl 1 reset cmd:ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>MISSING_LOGIC_NOTE</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>X61</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Logic note is empty.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>13OutPwm.csv</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E5"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
refactor: rename validation output to check sheet
</commit_message>
<xml_diff>
--- a/output/io_list_report.xlsx
+++ b/output/io_list_report.xlsx
@@ -10,12 +10,12 @@
     <sheet name="SUMMARY" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="INPUT" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="OUTPUT" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="ERROR" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="CHECK" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'INPUT'!$A$1:$H$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'OUTPUT'!$A$1:$H$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'ERROR'!$A$1:$E$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CHECK'!$A$1:$E$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -491,7 +491,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Warnings</t>
+          <t>Check items</t>
         </is>
       </c>
       <c r="B6" t="n">

</xml_diff>

<commit_message>
feat: merge device comments into IO report
</commit_message>
<xml_diff>
--- a/output/io_list_report.xlsx
+++ b/output/io_list_report.xlsx
@@ -13,9 +13,9 @@
     <sheet name="CHECK" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'INPUT'!$A$1:$H$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'OUTPUT'!$A$1:$H$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CHECK'!$A$1:$E$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'INPUT'!$A$1:$I$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'OUTPUT'!$A$1:$I$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CHECK'!$A$1:$E$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -451,7 +451,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Source CSV files</t>
+          <t>Ladder CSV files</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -461,41 +461,51 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Input devices</t>
+          <t>Device comments</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>22</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Output devices</t>
+          <t>Input devices</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Total devices</t>
+          <t>Output devices</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Total devices</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>Check items</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>4</v>
+      <c r="B7" t="n">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -509,17 +519,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="65" customWidth="1" min="7" max="7"/>
-    <col width="31" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="65" customWidth="1" min="8" max="8"/>
+    <col width="31" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -540,25 +551,30 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>DeviceComment</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>AddressNo</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>UsedFiles</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Instructions</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>LogicNotes</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Steps</t>
         </is>
@@ -578,25 +594,30 @@
           <t>X50</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>CH1 count start signal</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
         <v>80</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>01CmnPgm.csv</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>Count enable command:ON</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>01CmnPgm.csv:129</t>
         </is>
@@ -616,25 +637,30 @@
           <t>X51</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>CH1 count stop signal</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
         <v>81</v>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>01CmnPgm.csv</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>Count enable command:OFF</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>01CmnPgm.csv:145</t>
         </is>
@@ -654,25 +680,30 @@
           <t>X52</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>CH1 current value read signal</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
         <v>82</v>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>01CmnPgm.csv</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
       <c r="G4" t="inlineStr">
         <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
           <t>Stores current value in D2000</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>01CmnPgm.csv:161</t>
         </is>
@@ -692,25 +723,30 @@
           <t>X53</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>CH1 preset command signal</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
         <v>83</v>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>02PreSet.csv</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
       <c r="G5" t="inlineStr">
         <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
           <t>Preset command</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>02PreSet.csv:52</t>
         </is>
@@ -730,25 +766,30 @@
           <t>X54</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>CH1 counter fnc exe start signal</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
         <v>84</v>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>06DisCnt.csv</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
       <c r="G6" t="inlineStr">
         <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
           <t>Selected cnt fnc start cmd:ON</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>06DisCnt.csv:55</t>
         </is>
@@ -768,25 +809,30 @@
           <t>X55</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>CH1 counter fnc exe stop signal</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
         <v>85</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>06DisCnt.csv</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
       <c r="G7" t="inlineStr">
         <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
           <t>Selected cnt fnc start cmd:OFF</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>06DisCnt.csv:74</t>
         </is>
@@ -806,25 +852,30 @@
           <t>X56</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>CH1 latch 1 execution cmd signal</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
         <v>86</v>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>04Lcnt1.csv</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
       <c r="G8" t="inlineStr">
         <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
           <t>Selected counter fnc start cmd</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>04Lcnt1.csv:52</t>
         </is>
@@ -844,25 +895,30 @@
           <t>X57</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>CH1 latch cnt data 1 read signal</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
         <v>87</v>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>04Lcnt1.csv,08LcPre.csv</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
       <c r="G9" t="inlineStr">
         <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
           <t>Stores latch cnt val 1 in D2002,Stores latch cnt value in D2002</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>04Lcnt1.csv:71,08LcPre.csv:61</t>
         </is>
@@ -882,25 +938,30 @@
           <t>X58</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>CH1 latch cnt data 2 read signal</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
         <v>88</v>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>05Lcnt2.csv</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
       <c r="G10" t="inlineStr">
         <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
           <t>Stores latch cnt val 2 in D2004</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>05Lcnt2.csv:52</t>
         </is>
@@ -920,25 +981,30 @@
           <t>X59</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>CH1 sampling count start signal</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
         <v>89</v>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>07SplCnt.csv</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
       <c r="G11" t="inlineStr">
         <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
           <t>Selected counter fnc start cmd</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>07SplCnt.csv:57</t>
         </is>
@@ -958,25 +1024,30 @@
           <t>X5A</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>CH1 sampling cnt data read signl</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
         <v>90</v>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>07SplCnt.csv</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
       <c r="G12" t="inlineStr">
         <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
           <t>Stores sampling cnt val in D2006</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>07SplCnt.csv:76</t>
         </is>
@@ -996,25 +1067,30 @@
           <t>X5B</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>CH1 coinc output enable signal</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
         <v>91</v>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>03MchOut.csv</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
       <c r="G13" t="inlineStr">
         <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
           <t>Coincidence output enable cmd</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>03MchOut.csv:58</t>
         </is>
@@ -1034,25 +1110,30 @@
           <t>X5C</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>CH1 coincidence LED clear signal</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
         <v>92</v>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>03MchOut.csv</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>AND</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>Coinc sgnl 1 reset cmd:OFF,Coinc sgnl 1 reset cmd:ON</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>03MchOut.csv:98</t>
         </is>
@@ -1072,25 +1153,30 @@
           <t>X5D</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>CH1 freq measurement cmd signal</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
         <v>93</v>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>10ChkFrq.csv</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
       <c r="G15" t="inlineStr">
         <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
           <t>Stores measured freq in D2008</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>10ChkFrq.csv:57</t>
         </is>
@@ -1110,25 +1196,30 @@
           <t>X5E</t>
         </is>
       </c>
-      <c r="D16" t="n">
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>CH1 rot speed measure cmd signal</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
         <v>94</v>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>11ChkRsp.csv</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
       <c r="G16" t="inlineStr">
         <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
           <t>Stores measured rot spd in D2010</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>11ChkRsp.csv:58</t>
         </is>
@@ -1148,25 +1239,30 @@
           <t>X5F</t>
         </is>
       </c>
-      <c r="D17" t="n">
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>CH1 pulse measurement cmd signal</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
         <v>95</v>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>12ChkPls.csv</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
       <c r="G17" t="inlineStr">
         <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
           <t>Pulse measurement start command</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>12ChkPls.csv:55</t>
         </is>
@@ -1186,25 +1282,30 @@
           <t>X60</t>
         </is>
       </c>
-      <c r="D18" t="n">
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>CH1 measured pulse read signal</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
         <v>96</v>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>12ChkPls.csv</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
       <c r="G18" t="inlineStr">
         <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
           <t>Stores measured pulse in D2012</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>12ChkPls.csv:75</t>
         </is>
@@ -1224,21 +1325,26 @@
           <t>X61</t>
         </is>
       </c>
-      <c r="D19" t="n">
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>CH1 PWM output command signal</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
         <v>97</v>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>13OutPwm.csv</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr">
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
         <is>
           <t>13OutPwm.csv:86</t>
         </is>
@@ -1258,25 +1364,30 @@
           <t>X62</t>
         </is>
       </c>
-      <c r="D20" t="n">
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>CH1 error reset command signal</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
         <v>98</v>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>14RstErr.csv</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
       <c r="G20" t="inlineStr">
         <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
           <t>CH1 error reset command</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>14RstErr.csv:103</t>
         </is>
@@ -1296,25 +1407,26 @@
           <t>X97</t>
         </is>
       </c>
-      <c r="D21" t="n">
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="n">
         <v>151</v>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>99TestWarnging.csv</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
       <c r="G21" t="inlineStr">
         <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
           <t>Stores current value in D2000</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>99TestWarnging.csv:161</t>
         </is>
@@ -1334,25 +1446,26 @@
           <t>X98</t>
         </is>
       </c>
-      <c r="D22" t="n">
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="n">
         <v>152</v>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>99TestWarnging.csv</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
       <c r="G22" t="inlineStr">
         <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
           <t>Count enable command:OFF</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>99TestWarnging.csv:145</t>
         </is>
@@ -1372,32 +1485,33 @@
           <t>X99</t>
         </is>
       </c>
-      <c r="D23" t="n">
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="n">
         <v>153</v>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>99TestWarnging.csv</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
       <c r="G23" t="inlineStr">
         <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
           <t>Count enable command:ON</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>99TestWarnging.csv:129</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H23"/>
+  <autoFilter ref="A1:I23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1408,17 +1522,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1439,25 +1554,30 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>DeviceComment</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>AddressNo</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>UsedFiles</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Instructions</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>LogicNotes</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Steps</t>
         </is>
@@ -1477,25 +1597,30 @@
           <t>Y70</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>CH1 coinc confirmation LED sig</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
         <v>112</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>03MchOut.csv</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>OUT</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Coincidence conf LED signal</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>03MchOut.csv:80</t>
         </is>
@@ -1515,32 +1640,37 @@
           <t>Y71</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>CH1 ovrflw occurrence LED signal</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
         <v>113</v>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>09ChkOvr.csv</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>OUT</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Overflow confirmation LED signal</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>09ChkOvr.csv:59</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H3"/>
+  <autoFilter ref="A1:I3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1551,11 +1681,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="35" customWidth="1" min="4" max="4"/>
     <col width="65" customWidth="1" min="5" max="5"/>
@@ -1696,8 +1826,89 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>MISSING_DEVICE_COMMENT</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>X97</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Device comment is empty.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>99TestWarnging.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>MISSING_DEVICE_COMMENT</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>X98</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Device comment is empty.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>99TestWarnging.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>MISSING_DEVICE_COMMENT</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>X99</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Device comment is empty.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>99TestWarnging.csv</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E5"/>
+  <autoFilter ref="A1:E8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add raw data sheet and refresh project docs
</commit_message>
<xml_diff>
--- a/output/io_list_report.xlsx
+++ b/output/io_list_report.xlsx
@@ -11,11 +11,13 @@
     <sheet name="INPUT" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="OUTPUT" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="CHECK" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="RAW_DATA" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'INPUT'!$A$1:$I$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'INPUT'!$A$1:$I$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'OUTPUT'!$A$1:$I$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CHECK'!$A$1:$E$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CHECK'!$A$1:$E$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'RAW_DATA'!$A$1:$F$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -455,7 +457,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
@@ -475,7 +477,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5">
@@ -495,7 +497,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7">
@@ -505,7 +507,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -519,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1393,125 +1395,8 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>INPUT</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>X97</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="n">
-        <v>151</v>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>99TestWarnging.csv</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>Stores current value in D2000</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>99TestWarnging.csv:161</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>INPUT</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>X98</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="n">
-        <v>152</v>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>99TestWarnging.csv</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>Count enable command:OFF</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>99TestWarnging.csv:145</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>INPUT</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>X99</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="n">
-        <v>153</v>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>99TestWarnging.csv</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>Count enable command:ON</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>99TestWarnging.csv:129</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I23"/>
+  <autoFilter ref="A1:I20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1681,11 +1566,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="35" customWidth="1" min="4" max="4"/>
     <col width="65" customWidth="1" min="5" max="5"/>
@@ -1826,89 +1711,635 @@
         </is>
       </c>
     </row>
+  </sheetData>
+  <autoFilter ref="A1:E5"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SourceFile</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>RowNumber</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Instruction</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>LogicNote</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>19</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>129</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>X50</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>22</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>145</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>X51</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>25</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>161</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>X52</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>02PreSet.csv</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>X53</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+    </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>MISSING_DEVICE_COMMENT</t>
-        </is>
+          <t>03MchOut.csv</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>8</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>X97</t>
+          <t>58</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Device comment is empty.</t>
+          <t>LD</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>99TestWarnging.csv</t>
-        </is>
-      </c>
+          <t>X5B</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>MISSING_DEVICE_COMMENT</t>
-        </is>
+          <t>03MchOut.csv</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>14</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>X98</t>
+          <t>80</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Device comment is empty.</t>
+          <t>OUT</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>99TestWarnging.csv</t>
-        </is>
-      </c>
+          <t>Y70</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>MISSING_DEVICE_COMMENT</t>
-        </is>
+          <t>03MchOut.csv</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>17</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>X99</t>
+          <t>98</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Device comment is empty.</t>
+          <t>AND</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>99TestWarnging.csv</t>
-        </is>
-      </c>
+          <t>X5C</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>04Lcnt1.csv</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>X56</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>04Lcnt1.csv</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>11</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>X57</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>05Lcnt2.csv</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>8</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>X58</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>06DisCnt.csv</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>8</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>X54</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>06DisCnt.csv</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>11</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>X55</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>07SplCnt.csv</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>8</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>X59</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>07SplCnt.csv</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>11</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>X5A</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>08LcPre.csv</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>8</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>X57</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>09ChkOvr.csv</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>10</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Y71</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>10ChkFrq.csv</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>8</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>X5D</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>11ChkRsp.csv</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>8</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>X5E</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>12ChkPls.csv</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>8</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>X5F</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>12ChkPls.csv</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>11</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>X60</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>13OutPwm.csv</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>9</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>X61</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>14RstErr.csv</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>24</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>103</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>X62</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E8"/>
+  <autoFilter ref="A1:F23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: categorize check report items
</commit_message>
<xml_diff>
--- a/output/io_list_report.xlsx
+++ b/output/io_list_report.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'INPUT'!$A$1:$I$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'OUTPUT'!$A$1:$I$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CHECK'!$A$1:$E$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CHECK'!$A$1:$F$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'RAW_DATA'!$A$1:$F$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1566,14 +1566,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="65" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="80" customWidth="1" min="5" max="5"/>
+    <col width="65" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1584,20 +1585,25 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Message</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
@@ -1611,20 +1617,25 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Usage</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>MULTIPLE_USED_FILES</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>X57</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Device is used in multiple files.</t>
-        </is>
-      </c>
       <c r="E2" t="inlineStr">
+        <is>
+          <t>This I/O device is referenced in multiple ladder CSV files. Check whether the shared usage is intentional.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
         <is>
           <t>04Lcnt1.csv,08LcPre.csv</t>
         </is>
@@ -1638,20 +1649,25 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>LogicContext</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>MULTIPLE_LOGIC_NOTES</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>X57</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Device has multiple logic notes.</t>
-        </is>
-      </c>
       <c r="E3" t="inlineStr">
+        <is>
+          <t>Multiple logic notes were linked to this device. Review the context before using them as signal descriptions.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>Stores latch cnt val 1 in D2002,Stores latch cnt value in D2002</t>
         </is>
@@ -1665,20 +1681,25 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>LogicContext</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>MULTIPLE_LOGIC_NOTES</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>X5C</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Device has multiple logic notes.</t>
-        </is>
-      </c>
       <c r="E4" t="inlineStr">
+        <is>
+          <t>Multiple logic notes were linked to this device. Review the context before using them as signal descriptions.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>Coinc sgnl 1 reset cmd:OFF,Coinc sgnl 1 reset cmd:ON</t>
         </is>
@@ -1687,32 +1708,37 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>WARN</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>LogicContext</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>MISSING_LOGIC_NOTE</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>X61</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Logic note is empty.</t>
-        </is>
-      </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>No nearby ladder logic note was found for this device.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>13OutPwm.csv</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E5"/>
+  <autoFilter ref="A1:F5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: improve check report readability
</commit_message>
<xml_diff>
--- a/output/io_list_report.xlsx
+++ b/output/io_list_report.xlsx
@@ -38,7 +38,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -48,6 +48,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9EAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -63,9 +68,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -508,6 +515,36 @@
       </c>
       <c r="B7" t="n">
         <v>4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Check ERROR</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Check WARN</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Check INFO</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1610,128 +1647,128 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>WARN</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>LogicContext</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>MULTIPLE_LOGIC_NOTES</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>X57</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Multiple logic notes were linked to this device. Review the context before using them as signal descriptions.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Stores latch cnt val 1 in D2002,Stores latch cnt value in D2002</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>LogicContext</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>MULTIPLE_LOGIC_NOTES</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>X5C</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Multiple logic notes were linked to this device. Review the context before using them as signal descriptions.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Coinc sgnl 1 reset cmd:OFF,Coinc sgnl 1 reset cmd:ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Usage</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>MULTIPLE_USED_FILES</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>X57</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>This I/O device is referenced in multiple ladder CSV files. Check whether the shared usage is intentional.</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>04Lcnt1.csv,08LcPre.csv</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>LogicContext</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>MULTIPLE_LOGIC_NOTES</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>X57</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Multiple logic notes were linked to this device. Review the context before using them as signal descriptions.</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Stores latch cnt val 1 in D2002,Stores latch cnt value in D2002</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>WARN</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>LogicContext</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>MULTIPLE_LOGIC_NOTES</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>X5C</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Multiple logic notes were linked to this device. Review the context before using them as signal descriptions.</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Coinc sgnl 1 reset cmd:OFF,Coinc sgnl 1 reset cmd:ON</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>LogicContext</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>MISSING_LOGIC_NOTE</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>X61</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>No nearby ladder logic note was found for this device.</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>13OutPwm.csv</t>
         </is>

</xml_diff>

<commit_message>
feat: add device usage sheet
</commit_message>
<xml_diff>
--- a/output/io_list_report.xlsx
+++ b/output/io_list_report.xlsx
@@ -11,13 +11,15 @@
     <sheet name="INPUT" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="OUTPUT" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="CHECK" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="RAW_DATA" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="DEVICE_USAGE" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="RAW_DATA" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'INPUT'!$A$1:$I$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'OUTPUT'!$A$1:$I$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CHECK'!$A$1:$F$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'RAW_DATA'!$A$1:$F$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'DEVICE_USAGE'!$A$1:$G$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'RAW_DATA'!$A$1:$F$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -438,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -510,40 +512,50 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Check items</t>
+          <t>Device usage rows</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Check ERROR</t>
+          <t>Check items</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Check WARN</t>
+          <t>Check ERROR</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Check WARN</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Check INFO</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1786,6 +1798,1982 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G60"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="39" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>DeviceType</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Occurrences</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>UsedFiles</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Instructions</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Locations</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>D20</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>15Match.csv</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>IMASK</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>15Match.csv:row11,15Match.csv:row12:step64</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>D21</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>15Match.csv</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>INC</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>15Match.csv:row17:step70</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>D2000</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv:row27</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>D2002</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>04Lcnt1.csv,08LcPre.csv</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>04Lcnt1.csv:row13,08LcPre.csv:row10</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>D2004</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>05Lcnt2.csv</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>05Lcnt2.csv:row10</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>D2006</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>07SplCnt.csv</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>ICSMPRD1</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>07SplCnt.csv:row12:step77</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>D2008</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>10ChkFrq.csv</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>ICFCNT1</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>10ChkFrq.csv:row9:step58</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>D2010</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>11ChkRsp.csv</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>ICRCNT1</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>11ChkRsp.csv:row9:step59</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>D2012</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>12ChkPls.csv</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>ICPLSRD1</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>12ChkPls.csv:row12:step76</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>D2014</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>14RstErr.csv</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>14RstErr.csv:row14</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>D2015</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>14RstErr.csv</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>14RstErr.csv:row22</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>D2020</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>14RstErr.csv</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>AND&lt;&gt;,MOV</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>14RstErr.csv:row10,14RstErr.csv:row11:step59,14RstErr.csv:row13:step62</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>D2021</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>14RstErr.csv</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>AND&lt;&gt;,MOV</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>14RstErr.csv:row18,14RstErr.csv:row19:step82,14RstErr.csv:row21:step85</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>15Match.csv</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>MOV</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>15Match.csv:row10:step62</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>K-30000</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>ICRNGWR1</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv:row11:step69</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>K0</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>14RstErr.csv</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>14RstErr.csv:row12,14RstErr.csv:row20</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>K1</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>3</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv,04Lcnt1.csv,08LcPre.csv</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>ICCOVWR1,ICLTHRD1</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv:row14:step91,04Lcnt1.csv:row12:step72,08LcPre.csv:row9:step62</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>K2</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>05Lcnt2.csv</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>ICLTHRD1</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>05Lcnt2.csv:row9:step53</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>K1000</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv,13OutPwm.csv</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>ICPREWR1,ICPWM1</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv:row15,01CmnPgm.csv:row9:step54,13OutPwm.csv:row10:step87</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>K2000</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>13OutPwm.csv</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>13OutPwm.csv:row11</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>K30000</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv:row12</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>SD1880</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>DMOV</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv:row26:step162</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>SD1887</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>14RstErr.csv</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>MOV</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>14RstErr.csv:row9:step57</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>SD1888</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>14RstErr.csv</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>MOV</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>14RstErr.csv:row17:step80</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>SM</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>SM402</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv,15Match.csv</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv:row8:step53,15Match.csv:row9:step61</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>SM</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>SM1890</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>5</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv,03MchOut.csv</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>AND,ANI,RST,SET</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv:row17:step113,03MchOut.csv:row13:step79,03MchOut.csv:row18:step99,03MchOut.csv:row21:step116,03MchOut.csv:row22:step117</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>SM</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>SM1895</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>RST,SET</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv:row20:step130,01CmnPgm.csv:row23:step146</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>SM</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>SM1893</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>02PreSet.csv</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>02PreSet.csv:row9:step53</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>SM</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>SM1892</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>03MchOut.csv</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>LD,OUT</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>03MchOut.csv:row11:step77,03MchOut.csv:row9:step59</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>SM</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>SM1881</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>3</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>03MchOut.csv</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>AND,LD,LDI</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>03MchOut.csv:row12:step78,03MchOut.csv:row16:step97,03MchOut.csv:row20:step115</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>SM</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>SM1896</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>4</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>04Lcnt1.csv,06DisCnt.csv,07SplCnt.csv</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>OUT,RST,SET</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>04Lcnt1.csv:row9:step53,06DisCnt.csv:row12:step75,06DisCnt.csv:row9:step56,07SplCnt.csv:row9:step58</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>SD1882.1</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>09ChkOvr.csv</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>09ChkOvr.csv:row8:step57</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>SD1882.2</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>09ChkOvr.csv</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>09ChkOvr.csv:row9:step58</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>SM</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>SM1898</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>12ChkPls.csv</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>12ChkPls.csv:row9:step56</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>SM</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>SM1887</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>2</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>14RstErr.csv</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>14RstErr.csv:row25:step104,14RstErr.csv:row8:step56</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>SM</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>SM1888</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>2</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>14RstErr.csv</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>LD,OR</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>14RstErr.csv:row16:step79,14RstErr.csv:row26:step105</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>SM</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>SM1899</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>14RstErr.csv</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>14RstErr.csv:row28:step107</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>SM</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>SM400</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>15Match.csv</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>15Match.csv:row16:step69</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>X50</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv:row19:step129</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>X51</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv:row22:step145</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>X52</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv:row25:step161</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>X53</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>02PreSet.csv</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>02PreSet.csv:row8:step52</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>X54</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>06DisCnt.csv</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>06DisCnt.csv:row8:step55</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>X55</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>1</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>06DisCnt.csv</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>06DisCnt.csv:row11:step74</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>X56</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>04Lcnt1.csv</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>04Lcnt1.csv:row8:step52</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>X57</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>2</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>04Lcnt1.csv,08LcPre.csv</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>04Lcnt1.csv:row11:step71,08LcPre.csv:row8:step61</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>X58</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>1</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>05Lcnt2.csv</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>05Lcnt2.csv:row8:step52</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>X59</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>07SplCnt.csv</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>07SplCnt.csv:row8:step57</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>X5A</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>07SplCnt.csv</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>07SplCnt.csv:row11:step76</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>X5B</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>03MchOut.csv</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>03MchOut.csv:row8:step58</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>X5C</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>03MchOut.csv</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>AND</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>03MchOut.csv:row17:step98</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>X5D</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>10ChkFrq.csv</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>10ChkFrq.csv:row8:step57</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>X5E</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>11ChkRsp.csv</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>11ChkRsp.csv:row8:step58</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>X5F</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>12ChkPls.csv</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>12ChkPls.csv:row8:step55</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>X60</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>12ChkPls.csv</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>12ChkPls.csv:row11:step75</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>X61</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>13OutPwm.csv</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>13OutPwm.csv:row9:step86</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>X62</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>1</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>14RstErr.csv</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>14RstErr.csv:row24:step103</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Y70</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>03MchOut.csv</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>03MchOut.csv:row14:step80</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Y71</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>1</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>09ChkOvr.csv</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>09ChkOvr.csv:row10:step59</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G60"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
feat: add PLC reference sheets
</commit_message>
<xml_diff>
--- a/output/io_list_report.xlsx
+++ b/output/io_list_report.xlsx
@@ -12,14 +12,18 @@
     <sheet name="OUTPUT" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="CHECK" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="DEVICE_USAGE" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="RAW_DATA" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="INSTRUCTION_REFERENCE" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="DEVICE_TYPE_REFERENCE" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="RAW_DATA" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'INPUT'!$A$1:$I$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'OUTPUT'!$A$1:$I$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CHECK'!$A$1:$F$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'DEVICE_USAGE'!$A$1:$G$60</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'RAW_DATA'!$A$1:$F$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'INSTRUCTION_REFERENCE'!$A$1:$D$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'DEVICE_TYPE_REFERENCE'!$A$1:$D$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'RAW_DATA'!$A$1:$F$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3774,6 +3778,532 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="68" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Instruction</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>LadderExample</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Load</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>|--[ X0 ]--</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Starts a condition using a normally open contact.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AND</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>And</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>|--[ X0 ]--[ X1 ]--</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Adds a serial condition. All serial conditions must be true.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Or</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Parallel branch</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Adds a parallel condition. Any branch can make the condition true.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ANI</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>And Not</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>|--[ X0 ]--[/ X1 ]--</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Adds a serial normally closed condition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>|--[ X0 ]--( Y0 )--</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Writes the condition result to an output coil or internal bit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SET</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Set</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>|--[ X0 ]--( SET M0 )--</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Turns a bit on and keeps it on until it is reset.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>RST</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Reset</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>|--[ X1 ]--( RST M0 )--</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Turns a set bit off.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MOV</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Move</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MOV D0 D10</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Copies a value from a source device to a destination device.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DMOV</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Double Move</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>DMOV SD1880 D2000</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Copies a 32-bit value, usually using two consecutive words.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>INC</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Increment</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>INC D0</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Increases the target device value by one.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="72" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>DeviceType</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Example</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>X0</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Physical input such as a sensor, push button, or switch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Y0</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Physical output such as a lamp, relay, solenoid, or actuator signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Internal relay</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>M100</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Internal bit used inside the PLC program.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SM</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Special relay</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>SM402</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>System bit provided by the PLC CPU or special function area.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Data register</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>D2000</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Word register used to store numeric values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Special data register</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>SD1880</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>System data register provided by the PLC CPU or special function area.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Decimal constant</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>K1000</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Fixed decimal value used as an instruction parameter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Hex constant</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Fixed hexadecimal value used as an instruction parameter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Timer</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Timer device used for time-based control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Counter</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>C0</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Counter device used for count-based control.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
refactor: exclude IO devices from device usage sheet
</commit_message>
<xml_diff>
--- a/output/io_list_report.xlsx
+++ b/output/io_list_report.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'INPUT'!$A$1:$I$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'OUTPUT'!$A$1:$I$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CHECK'!$A$1:$F$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'DEVICE_USAGE'!$A$1:$G$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'DEVICE_USAGE'!$A$1:$G$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'INSTRUCTION_REFERENCE'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'DEVICE_TYPE_REFERENCE'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'RAW_DATA'!$A$1:$F$23</definedName>
@@ -520,7 +520,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>59</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8">
@@ -1802,7 +1802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G60"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3073,701 +3073,8 @@
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="n">
-        <v>39</v>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>X50</t>
-        </is>
-      </c>
-      <c r="D40" t="n">
-        <v>1</v>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>01CmnPgm.csv</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>01CmnPgm.csv:row19:step129</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="n">
-        <v>40</v>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>X51</t>
-        </is>
-      </c>
-      <c r="D41" t="n">
-        <v>1</v>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>01CmnPgm.csv</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>01CmnPgm.csv:row22:step145</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="n">
-        <v>41</v>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>X52</t>
-        </is>
-      </c>
-      <c r="D42" t="n">
-        <v>1</v>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>01CmnPgm.csv</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>01CmnPgm.csv:row25:step161</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
-        <v>42</v>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>X53</t>
-        </is>
-      </c>
-      <c r="D43" t="n">
-        <v>1</v>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>02PreSet.csv</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>02PreSet.csv:row8:step52</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="n">
-        <v>43</v>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>X54</t>
-        </is>
-      </c>
-      <c r="D44" t="n">
-        <v>1</v>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>06DisCnt.csv</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>06DisCnt.csv:row8:step55</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="n">
-        <v>44</v>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>X55</t>
-        </is>
-      </c>
-      <c r="D45" t="n">
-        <v>1</v>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>06DisCnt.csv</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>06DisCnt.csv:row11:step74</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="n">
-        <v>45</v>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>X56</t>
-        </is>
-      </c>
-      <c r="D46" t="n">
-        <v>1</v>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>04Lcnt1.csv</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>04Lcnt1.csv:row8:step52</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="n">
-        <v>46</v>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>X57</t>
-        </is>
-      </c>
-      <c r="D47" t="n">
-        <v>2</v>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>04Lcnt1.csv,08LcPre.csv</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>04Lcnt1.csv:row11:step71,08LcPre.csv:row8:step61</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="n">
-        <v>47</v>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>X58</t>
-        </is>
-      </c>
-      <c r="D48" t="n">
-        <v>1</v>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>05Lcnt2.csv</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>05Lcnt2.csv:row8:step52</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="n">
-        <v>48</v>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>X59</t>
-        </is>
-      </c>
-      <c r="D49" t="n">
-        <v>1</v>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>07SplCnt.csv</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>07SplCnt.csv:row8:step57</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="n">
-        <v>49</v>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>X5A</t>
-        </is>
-      </c>
-      <c r="D50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>07SplCnt.csv</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>07SplCnt.csv:row11:step76</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="n">
-        <v>50</v>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>X5B</t>
-        </is>
-      </c>
-      <c r="D51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>03MchOut.csv</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>03MchOut.csv:row8:step58</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="n">
-        <v>51</v>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>X5C</t>
-        </is>
-      </c>
-      <c r="D52" t="n">
-        <v>1</v>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>03MchOut.csv</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>AND</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>03MchOut.csv:row17:step98</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="n">
-        <v>52</v>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>X5D</t>
-        </is>
-      </c>
-      <c r="D53" t="n">
-        <v>1</v>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>10ChkFrq.csv</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>10ChkFrq.csv:row8:step57</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="n">
-        <v>53</v>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>X5E</t>
-        </is>
-      </c>
-      <c r="D54" t="n">
-        <v>1</v>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>11ChkRsp.csv</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>11ChkRsp.csv:row8:step58</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="n">
-        <v>54</v>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>X5F</t>
-        </is>
-      </c>
-      <c r="D55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>12ChkPls.csv</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>12ChkPls.csv:row8:step55</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="n">
-        <v>55</v>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>X60</t>
-        </is>
-      </c>
-      <c r="D56" t="n">
-        <v>1</v>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>12ChkPls.csv</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>12ChkPls.csv:row11:step75</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="n">
-        <v>56</v>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>X61</t>
-        </is>
-      </c>
-      <c r="D57" t="n">
-        <v>1</v>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>13OutPwm.csv</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>13OutPwm.csv:row9:step86</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="n">
-        <v>57</v>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>X62</t>
-        </is>
-      </c>
-      <c r="D58" t="n">
-        <v>1</v>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>14RstErr.csv</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>14RstErr.csv:row24:step103</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="n">
-        <v>58</v>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Y70</t>
-        </is>
-      </c>
-      <c r="D59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>03MchOut.csv</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>03MchOut.csv:row14:step80</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="n">
-        <v>59</v>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Y71</t>
-        </is>
-      </c>
-      <c r="D60" t="n">
-        <v>1</v>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>09ChkOvr.csv</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>09ChkOvr.csv:row10:step59</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G60"/>
+  <autoFilter ref="A1:G39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs: rewrite README for project scope and usage
</commit_message>
<xml_diff>
--- a/output/io_list_report.xlsx
+++ b/output/io_list_report.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'INPUT'!$A$1:$I$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'OUTPUT'!$A$1:$I$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CHECK'!$A$1:$F$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'DEVICE_USAGE'!$A$1:$G$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'DEVICE_USAGE'!$A$1:$H$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'INSTRUCTION_REFERENCE'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'DEVICE_TYPE_REFERENCE'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'RAW_DATA'!$A$1:$F$23</definedName>
@@ -1802,16 +1802,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="39" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
-    <col width="80" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="39" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="80" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1832,20 +1833,25 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>DeviceComment</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Occurrences</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>UsedFiles</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Instructions</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Locations</t>
         </is>
@@ -1865,20 +1871,25 @@
           <t>D20</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>IMASK instruct intp enable flag</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
         <v>2</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>15Match.csv</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>IMASK</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>15Match.csv:row11,15Match.csv:row12:step64</t>
         </is>
@@ -1898,20 +1909,21 @@
           <t>D21</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="n">
         <v>1</v>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>15Match.csv</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>INC</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>15Match.csv:row17:step70</t>
         </is>
@@ -1931,16 +1943,21 @@
           <t>D2000</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>CH1 current value (Lo 16 bit)</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
         <v>1</v>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>01CmnPgm.csv</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
         <is>
           <t>01CmnPgm.csv:row27</t>
         </is>
@@ -1960,16 +1977,21 @@
           <t>D2002</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>CH1 latch cnt val 1 (Lo 16 bit)</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
         <v>2</v>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>04Lcnt1.csv,08LcPre.csv</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
         <is>
           <t>04Lcnt1.csv:row13,08LcPre.csv:row10</t>
         </is>
@@ -1989,16 +2011,21 @@
           <t>D2004</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>CH1 latch cnt val 2 (Lo 16 bit)</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
         <v>1</v>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>05Lcnt2.csv</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
         <is>
           <t>05Lcnt2.csv:row10</t>
         </is>
@@ -2018,20 +2045,25 @@
           <t>D2006</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>CH1 sampling cnt val (Lo 16 bit)</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
         <v>1</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>07SplCnt.csv</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>ICSMPRD1</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>07SplCnt.csv:row12:step77</t>
         </is>
@@ -2051,20 +2083,25 @@
           <t>D2008</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>CH1 measur freq val (Lo 16 bit)</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
         <v>1</v>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>10ChkFrq.csv</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>ICFCNT1</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>10ChkFrq.csv:row9:step58</t>
         </is>
@@ -2084,20 +2121,25 @@
           <t>D2010</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>CH1 measur rot sp val (Lo 16B)</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
         <v>1</v>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>11ChkRsp.csv</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>ICRCNT1</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>11ChkRsp.csv:row9:step59</t>
         </is>
@@ -2117,20 +2159,25 @@
           <t>D2012</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>CH1 measured pul val (Lo 16 bit)</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
         <v>1</v>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>12ChkPls.csv</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>ICPLSRD1</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>12ChkPls.csv:row12:step76</t>
         </is>
@@ -2150,16 +2197,21 @@
           <t>D2014</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>CH1 error code storage</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
         <v>1</v>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>14RstErr.csv</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr">
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
         <is>
           <t>14RstErr.csv:row14</t>
         </is>
@@ -2179,16 +2231,21 @@
           <t>D2015</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>CH1 warning code storage</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
         <v>1</v>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>14RstErr.csv</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr">
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
         <is>
           <t>14RstErr.csv:row22</t>
         </is>
@@ -2208,20 +2265,25 @@
           <t>D2020</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>CH1 error code acquisition</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
         <v>3</v>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>14RstErr.csv</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>AND&lt;&gt;,MOV</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>14RstErr.csv:row10,14RstErr.csv:row11:step59,14RstErr.csv:row13:step62</t>
         </is>
@@ -2241,20 +2303,25 @@
           <t>D2021</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>CH1 warning code acquisition</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
         <v>3</v>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>14RstErr.csv</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>AND&lt;&gt;,MOV</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>14RstErr.csv:row18,14RstErr.csv:row19:step82,14RstErr.csv:row21:step85</t>
         </is>
@@ -2274,20 +2341,21 @@
           <t>H1</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="n">
         <v>1</v>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>15Match.csv</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>MOV</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>15Match.csv:row10:step62</t>
         </is>
@@ -2307,20 +2375,21 @@
           <t>K-30000</t>
         </is>
       </c>
-      <c r="D16" t="n">
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="n">
         <v>1</v>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>01CmnPgm.csv</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>ICRNGWR1</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>01CmnPgm.csv:row11:step69</t>
         </is>
@@ -2340,16 +2409,17 @@
           <t>K0</t>
         </is>
       </c>
-      <c r="D17" t="n">
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="n">
         <v>2</v>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>14RstErr.csv</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr">
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
         <is>
           <t>14RstErr.csv:row12,14RstErr.csv:row20</t>
         </is>
@@ -2369,20 +2439,21 @@
           <t>K1</t>
         </is>
       </c>
-      <c r="D18" t="n">
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="n">
         <v>3</v>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>01CmnPgm.csv,04Lcnt1.csv,08LcPre.csv</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>ICCOVWR1,ICLTHRD1</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>01CmnPgm.csv:row14:step91,04Lcnt1.csv:row12:step72,08LcPre.csv:row9:step62</t>
         </is>
@@ -2402,20 +2473,21 @@
           <t>K2</t>
         </is>
       </c>
-      <c r="D19" t="n">
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="n">
         <v>1</v>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>05Lcnt2.csv</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>ICLTHRD1</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>05Lcnt2.csv:row9:step53</t>
         </is>
@@ -2435,20 +2507,21 @@
           <t>K1000</t>
         </is>
       </c>
-      <c r="D20" t="n">
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="n">
         <v>3</v>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>01CmnPgm.csv,13OutPwm.csv</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>ICPREWR1,ICPWM1</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>01CmnPgm.csv:row15,01CmnPgm.csv:row9:step54,13OutPwm.csv:row10:step87</t>
         </is>
@@ -2468,16 +2541,17 @@
           <t>K2000</t>
         </is>
       </c>
-      <c r="D21" t="n">
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="n">
         <v>1</v>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>13OutPwm.csv</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr">
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
         <is>
           <t>13OutPwm.csv:row11</t>
         </is>
@@ -2497,16 +2571,17 @@
           <t>K30000</t>
         </is>
       </c>
-      <c r="D22" t="n">
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="n">
         <v>1</v>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>01CmnPgm.csv</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr">
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
         <is>
           <t>01CmnPgm.csv:row12</t>
         </is>
@@ -2526,20 +2601,25 @@
           <t>SD1880</t>
         </is>
       </c>
-      <c r="D23" t="n">
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>CH1 current value (Lo 16 bit)</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
         <v>1</v>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>01CmnPgm.csv</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>DMOV</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>01CmnPgm.csv:row26:step162</t>
         </is>
@@ -2559,20 +2639,25 @@
           <t>SD1887</t>
         </is>
       </c>
-      <c r="D24" t="n">
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>CH1 error code</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
         <v>1</v>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>14RstErr.csv</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>MOV</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>14RstErr.csv:row9:step57</t>
         </is>
@@ -2592,20 +2677,25 @@
           <t>SD1888</t>
         </is>
       </c>
-      <c r="D25" t="n">
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>CH1 warning code</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
         <v>1</v>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>14RstErr.csv</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>MOV</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>14RstErr.csv:row17:step80</t>
         </is>
@@ -2625,20 +2715,25 @@
           <t>SM402</t>
         </is>
       </c>
-      <c r="D26" t="n">
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Turned ON for one scan after RUN</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
         <v>2</v>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>01CmnPgm.csv,15Match.csv</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>LD</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>01CmnPgm.csv:row8:step53,15Match.csv:row9:step61</t>
         </is>
@@ -2658,20 +2753,25 @@
           <t>SM1890</t>
         </is>
       </c>
-      <c r="D27" t="n">
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>CH1 coinc signal 1 reset cmd</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
         <v>5</v>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>01CmnPgm.csv,03MchOut.csv</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>AND,ANI,RST,SET</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="H27" t="inlineStr">
         <is>
           <t>01CmnPgm.csv:row17:step113,03MchOut.csv:row13:step79,03MchOut.csv:row18:step99,03MchOut.csv:row21:step116,03MchOut.csv:row22:step117</t>
         </is>
@@ -2691,20 +2791,25 @@
           <t>SM1895</t>
         </is>
       </c>
-      <c r="D28" t="n">
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>CH1 counter enable command</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
         <v>2</v>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>01CmnPgm.csv</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>RST,SET</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>01CmnPgm.csv:row20:step130,01CmnPgm.csv:row23:step146</t>
         </is>
@@ -2724,20 +2829,25 @@
           <t>SM1893</t>
         </is>
       </c>
-      <c r="D29" t="n">
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>CH1 preset command</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
         <v>1</v>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>02PreSet.csv</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>OUT</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>02PreSet.csv:row9:step53</t>
         </is>
@@ -2757,20 +2867,25 @@
           <t>SM1892</t>
         </is>
       </c>
-      <c r="D30" t="n">
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>CH1 coinc output enable cmd</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
         <v>2</v>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>03MchOut.csv</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>LD,OUT</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>03MchOut.csv:row11:step77,03MchOut.csv:row9:step59</t>
         </is>
@@ -2790,20 +2905,25 @@
           <t>SM1881</t>
         </is>
       </c>
-      <c r="D31" t="n">
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>CH1 cnt value coinc No. 1</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
         <v>3</v>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>03MchOut.csv</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>AND,LD,LDI</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="H31" t="inlineStr">
         <is>
           <t>03MchOut.csv:row12:step78,03MchOut.csv:row16:step97,03MchOut.csv:row20:step115</t>
         </is>
@@ -2823,20 +2943,25 @@
           <t>SM1896</t>
         </is>
       </c>
-      <c r="D32" t="n">
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>CH1 sel cnt fnc start cmd</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
         <v>4</v>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>04Lcnt1.csv,06DisCnt.csv,07SplCnt.csv</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>OUT,RST,SET</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="H32" t="inlineStr">
         <is>
           <t>04Lcnt1.csv:row9:step53,06DisCnt.csv:row12:step75,06DisCnt.csv:row9:step56,07SplCnt.csv:row9:step58</t>
         </is>
@@ -2856,20 +2981,21 @@
           <t>SD1882.1</t>
         </is>
       </c>
-      <c r="D33" t="n">
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="n">
         <v>1</v>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>09ChkOvr.csv</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="G33" t="inlineStr">
         <is>
           <t>LD</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="H33" t="inlineStr">
         <is>
           <t>09ChkOvr.csv:row8:step57</t>
         </is>
@@ -2889,20 +3015,21 @@
           <t>SD1882.2</t>
         </is>
       </c>
-      <c r="D34" t="n">
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="n">
         <v>1</v>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>09ChkOvr.csv</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>OR</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="H34" t="inlineStr">
         <is>
           <t>09ChkOvr.csv:row9:step58</t>
         </is>
@@ -2922,20 +3049,25 @@
           <t>SM1898</t>
         </is>
       </c>
-      <c r="D35" t="n">
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>CH1 pulse measure start cmd</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
         <v>1</v>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>12ChkPls.csv</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="G35" t="inlineStr">
         <is>
           <t>OUT</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="H35" t="inlineStr">
         <is>
           <t>12ChkPls.csv:row9:step56</t>
         </is>
@@ -2955,20 +3087,25 @@
           <t>SM1887</t>
         </is>
       </c>
-      <c r="D36" t="n">
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>CH1 error</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
         <v>2</v>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>14RstErr.csv</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="G36" t="inlineStr">
         <is>
           <t>LD</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="H36" t="inlineStr">
         <is>
           <t>14RstErr.csv:row25:step104,14RstErr.csv:row8:step56</t>
         </is>
@@ -2988,20 +3125,25 @@
           <t>SM1888</t>
         </is>
       </c>
-      <c r="D37" t="n">
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>CH1 warning</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
         <v>2</v>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>14RstErr.csv</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>LD,OR</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="H37" t="inlineStr">
         <is>
           <t>14RstErr.csv:row16:step79,14RstErr.csv:row26:step105</t>
         </is>
@@ -3021,20 +3163,25 @@
           <t>SM1899</t>
         </is>
       </c>
-      <c r="D38" t="n">
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>CH1 error reset command</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
         <v>1</v>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>14RstErr.csv</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="G38" t="inlineStr">
         <is>
           <t>OUT</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="H38" t="inlineStr">
         <is>
           <t>14RstErr.csv:row28:step107</t>
         </is>
@@ -3054,27 +3201,32 @@
           <t>SM400</t>
         </is>
       </c>
-      <c r="D39" t="n">
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Always ON</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
         <v>1</v>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>15Match.csv</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="G39" t="inlineStr">
         <is>
           <t>LD</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="H39" t="inlineStr">
         <is>
           <t>15Match.csv:row16:step69</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G39"/>
+  <autoFilter ref="A1:H39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: categorize device usage rows
</commit_message>
<xml_diff>
--- a/output/io_list_report.xlsx
+++ b/output/io_list_report.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'INPUT'!$A$1:$I$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'OUTPUT'!$A$1:$I$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CHECK'!$A$1:$F$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'DEVICE_USAGE'!$A$1:$H$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'DEVICE_USAGE'!$A$1:$I$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'INSTRUCTION_REFERENCE'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'DEVICE_TYPE_REFERENCE'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'RAW_DATA'!$A$1:$F$23</definedName>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -466,100 +466,172 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ladder CSV files</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>15</v>
+          <t>Project name</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>LD-LCPU_CNT_V100A_E</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Device comments</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>57</v>
+          <t>Generated at</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:59:57</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Input devices</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>19</v>
+          <t>Ladder CSV folder</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>samples\ladder</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Output devices</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>2</v>
+          <t>Device comment file</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>samples\device_comments\device_comments.csv</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Total devices</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>21</v>
+          <t>Output CSV</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>output\io_list.csv</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Device usage rows</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>38</v>
+          <t>Output Excel</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>output\io_list_report.xlsx</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Check items</t>
+          <t>Ladder CSV files</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Check ERROR</t>
+          <t>Device comments</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Check WARN</t>
+          <t>Input devices</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>Output devices</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Total devices</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Device usage rows</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Check items</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Check ERROR</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Check WARN</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>Check INFO</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B17" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1802,17 +1874,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="39" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="80" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="39" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="80" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1823,35 +1896,40 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>UsageCategory</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>DeviceType</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>DeviceComment</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Occurrences</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>UsedFiles</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Instructions</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Locations</t>
         </is>
@@ -1863,33 +1941,38 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>InternalDevice</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>D20</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>IMASK instruct intp enable flag</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>2</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>15Match.csv</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>IMASK</t>
-        </is>
-      </c>
       <c r="H2" t="inlineStr">
+        <is>
+          <t>IMASK,MOV</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>15Match.csv:row11,15Match.csv:row12:step64</t>
         </is>
@@ -1901,29 +1984,34 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>InternalDevice</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>D21</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="n">
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="n">
         <v>1</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>15Match.csv</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>INC</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>15Match.csv:row17:step70</t>
         </is>
@@ -1935,29 +2023,38 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>InternalDevice</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>D2000</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>CH1 current value (Lo 16 bit)</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>1</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>01CmnPgm.csv</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
+        <is>
+          <t>DMOV</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
         <is>
           <t>01CmnPgm.csv:row27</t>
         </is>
@@ -1969,29 +2066,38 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>InternalDevice</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>D2002</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>CH1 latch cnt val 1 (Lo 16 bit)</t>
         </is>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>2</v>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>04Lcnt1.csv,08LcPre.csv</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
+        <is>
+          <t>ICLTHRD1</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
         <is>
           <t>04Lcnt1.csv:row13,08LcPre.csv:row10</t>
         </is>
@@ -2003,29 +2109,38 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>InternalDevice</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>D2004</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>CH1 latch cnt val 2 (Lo 16 bit)</t>
         </is>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>1</v>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>05Lcnt2.csv</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
+        <is>
+          <t>ICLTHRD1</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
         <is>
           <t>05Lcnt2.csv:row10</t>
         </is>
@@ -2037,33 +2152,38 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>InternalDevice</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>D2006</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>CH1 sampling cnt val (Lo 16 bit)</t>
         </is>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>1</v>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>07SplCnt.csv</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>ICSMPRD1</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>07SplCnt.csv:row12:step77</t>
         </is>
@@ -2075,33 +2195,38 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>InternalDevice</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>D2008</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>CH1 measur freq val (Lo 16 bit)</t>
         </is>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>1</v>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>10ChkFrq.csv</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>ICFCNT1</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>10ChkFrq.csv:row9:step58</t>
         </is>
@@ -2113,33 +2238,38 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>InternalDevice</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>D2010</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>CH1 measur rot sp val (Lo 16B)</t>
         </is>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>1</v>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>11ChkRsp.csv</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>ICRCNT1</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>11ChkRsp.csv:row9:step59</t>
         </is>
@@ -2151,33 +2281,38 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>InternalDevice</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>D2012</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>CH1 measured pul val (Lo 16 bit)</t>
         </is>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>1</v>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>12ChkPls.csv</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>ICPLSRD1</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>12ChkPls.csv:row12:step76</t>
         </is>
@@ -2189,29 +2324,38 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>InternalDevice</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>D2014</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>CH1 error code storage</t>
         </is>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>1</v>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>14RstErr.csv</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
+        <is>
+          <t>MOV</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
         <is>
           <t>14RstErr.csv:row14</t>
         </is>
@@ -2223,29 +2367,38 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>InternalDevice</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>D2015</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>CH1 warning code storage</t>
         </is>
       </c>
-      <c r="E12" t="n">
+      <c r="F12" t="n">
         <v>1</v>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>14RstErr.csv</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
+        <is>
+          <t>MOV</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
         <is>
           <t>14RstErr.csv:row22</t>
         </is>
@@ -2257,33 +2410,38 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>InternalDevice</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>D2020</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>CH1 error code acquisition</t>
         </is>
       </c>
-      <c r="E13" t="n">
+      <c r="F13" t="n">
         <v>3</v>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>14RstErr.csv</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>AND&lt;&gt;,MOV</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>14RstErr.csv:row10,14RstErr.csv:row11:step59,14RstErr.csv:row13:step62</t>
         </is>
@@ -2295,33 +2453,38 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>InternalDevice</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>D2021</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>CH1 warning code acquisition</t>
         </is>
       </c>
-      <c r="E14" t="n">
+      <c r="F14" t="n">
         <v>3</v>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>14RstErr.csv</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>AND&lt;&gt;,MOV</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>14RstErr.csv:row18,14RstErr.csv:row19:step82,14RstErr.csv:row21:step85</t>
         </is>
@@ -2333,29 +2496,34 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>Constant</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
           <t>H</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>H1</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="n">
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="n">
         <v>1</v>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>15Match.csv</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>MOV</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>15Match.csv:row10:step62</t>
         </is>
@@ -2367,29 +2535,34 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>Constant</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>K-30000</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="n">
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="n">
         <v>1</v>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>01CmnPgm.csv</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>ICRNGWR1</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>01CmnPgm.csv:row11:step69</t>
         </is>
@@ -2401,25 +2574,34 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>Constant</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>K0</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="n">
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="n">
         <v>2</v>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>14RstErr.csv</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
+        <is>
+          <t>AND&lt;&gt;</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
         <is>
           <t>14RstErr.csv:row12,14RstErr.csv:row20</t>
         </is>
@@ -2431,29 +2613,34 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>Constant</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>K1</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="n">
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="n">
         <v>3</v>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>01CmnPgm.csv,04Lcnt1.csv,08LcPre.csv</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>ICCOVWR1,ICLTHRD1</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>01CmnPgm.csv:row14:step91,04Lcnt1.csv:row12:step72,08LcPre.csv:row9:step62</t>
         </is>
@@ -2465,29 +2652,34 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t>Constant</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>K2</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="n">
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="n">
         <v>1</v>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>05Lcnt2.csv</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>ICLTHRD1</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>05Lcnt2.csv:row9:step53</t>
         </is>
@@ -2499,29 +2691,34 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>Constant</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>K1000</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="n">
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="n">
         <v>3</v>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>01CmnPgm.csv,13OutPwm.csv</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>ICPREWR1,ICPWM1</t>
-        </is>
-      </c>
       <c r="H20" t="inlineStr">
+        <is>
+          <t>ICCOVWR1,ICPREWR1,ICPWM1</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
         <is>
           <t>01CmnPgm.csv:row15,01CmnPgm.csv:row9:step54,13OutPwm.csv:row10:step87</t>
         </is>
@@ -2533,25 +2730,34 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>Constant</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>K2000</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="n">
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="n">
         <v>1</v>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>13OutPwm.csv</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
+        <is>
+          <t>ICPWM1</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
         <is>
           <t>13OutPwm.csv:row11</t>
         </is>
@@ -2563,25 +2769,34 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>Constant</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>K30000</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="n">
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="n">
         <v>1</v>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>01CmnPgm.csv</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
+        <is>
+          <t>ICRNGWR1</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
         <is>
           <t>01CmnPgm.csv:row12</t>
         </is>
@@ -2593,33 +2808,38 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
+          <t>SpecialDevice</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
           <t>SD</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>SD1880</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>CH1 current value (Lo 16 bit)</t>
         </is>
       </c>
-      <c r="E23" t="n">
+      <c r="F23" t="n">
         <v>1</v>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>01CmnPgm.csv</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>DMOV</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>01CmnPgm.csv:row26:step162</t>
         </is>
@@ -2631,33 +2851,38 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
+          <t>SpecialDevice</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
           <t>SD</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>SD1887</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>CH1 error code</t>
         </is>
       </c>
-      <c r="E24" t="n">
+      <c r="F24" t="n">
         <v>1</v>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>14RstErr.csv</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>MOV</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>14RstErr.csv:row9:step57</t>
         </is>
@@ -2669,33 +2894,38 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>SpecialDevice</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
           <t>SD</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>SD1888</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>CH1 warning code</t>
         </is>
       </c>
-      <c r="E25" t="n">
+      <c r="F25" t="n">
         <v>1</v>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>14RstErr.csv</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>MOV</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>14RstErr.csv:row17:step80</t>
         </is>
@@ -2707,33 +2937,38 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
+          <t>SpecialDevice</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
           <t>SM</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>SM402</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>Turned ON for one scan after RUN</t>
         </is>
       </c>
-      <c r="E26" t="n">
+      <c r="F26" t="n">
         <v>2</v>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>01CmnPgm.csv,15Match.csv</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>LD</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>01CmnPgm.csv:row8:step53,15Match.csv:row9:step61</t>
         </is>
@@ -2745,33 +2980,38 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
+          <t>SpecialDevice</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
           <t>SM</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>SM1890</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>CH1 coinc signal 1 reset cmd</t>
         </is>
       </c>
-      <c r="E27" t="n">
+      <c r="F27" t="n">
         <v>5</v>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>01CmnPgm.csv,03MchOut.csv</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="H27" t="inlineStr">
         <is>
           <t>AND,ANI,RST,SET</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="I27" t="inlineStr">
         <is>
           <t>01CmnPgm.csv:row17:step113,03MchOut.csv:row13:step79,03MchOut.csv:row18:step99,03MchOut.csv:row21:step116,03MchOut.csv:row22:step117</t>
         </is>
@@ -2783,33 +3023,38 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
+          <t>SpecialDevice</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
           <t>SM</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>SM1895</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>CH1 counter enable command</t>
         </is>
       </c>
-      <c r="E28" t="n">
+      <c r="F28" t="n">
         <v>2</v>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>01CmnPgm.csv</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>RST,SET</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t>01CmnPgm.csv:row20:step130,01CmnPgm.csv:row23:step146</t>
         </is>
@@ -2821,33 +3066,38 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
+          <t>SpecialDevice</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
           <t>SM</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>SM1893</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>CH1 preset command</t>
         </is>
       </c>
-      <c r="E29" t="n">
+      <c r="F29" t="n">
         <v>1</v>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>02PreSet.csv</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>OUT</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t>02PreSet.csv:row9:step53</t>
         </is>
@@ -2859,33 +3109,38 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
+          <t>SpecialDevice</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
           <t>SM</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>SM1892</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>CH1 coinc output enable cmd</t>
         </is>
       </c>
-      <c r="E30" t="n">
+      <c r="F30" t="n">
         <v>2</v>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>03MchOut.csv</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>LD,OUT</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t>03MchOut.csv:row11:step77,03MchOut.csv:row9:step59</t>
         </is>
@@ -2897,33 +3152,38 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
+          <t>SpecialDevice</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
           <t>SM</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>SM1881</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>CH1 cnt value coinc No. 1</t>
         </is>
       </c>
-      <c r="E31" t="n">
+      <c r="F31" t="n">
         <v>3</v>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>03MchOut.csv</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="H31" t="inlineStr">
         <is>
           <t>AND,LD,LDI</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="I31" t="inlineStr">
         <is>
           <t>03MchOut.csv:row12:step78,03MchOut.csv:row16:step97,03MchOut.csv:row20:step115</t>
         </is>
@@ -2935,33 +3195,38 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
+          <t>SpecialDevice</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
           <t>SM</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>SM1896</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>CH1 sel cnt fnc start cmd</t>
         </is>
       </c>
-      <c r="E32" t="n">
+      <c r="F32" t="n">
         <v>4</v>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>04Lcnt1.csv,06DisCnt.csv,07SplCnt.csv</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="H32" t="inlineStr">
         <is>
           <t>OUT,RST,SET</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="I32" t="inlineStr">
         <is>
           <t>04Lcnt1.csv:row9:step53,06DisCnt.csv:row12:step75,06DisCnt.csv:row9:step56,07SplCnt.csv:row9:step58</t>
         </is>
@@ -2973,29 +3238,34 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
+          <t>SpecialDevice</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
           <t>SD</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>SD1882.1</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="n">
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="n">
         <v>1</v>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="G33" t="inlineStr">
         <is>
           <t>09ChkOvr.csv</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="H33" t="inlineStr">
         <is>
           <t>LD</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="I33" t="inlineStr">
         <is>
           <t>09ChkOvr.csv:row8:step57</t>
         </is>
@@ -3007,29 +3277,34 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>SpecialDevice</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
           <t>SD</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>SD1882.2</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="n">
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="n">
         <v>1</v>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>09ChkOvr.csv</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="H34" t="inlineStr">
         <is>
           <t>OR</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="I34" t="inlineStr">
         <is>
           <t>09ChkOvr.csv:row9:step58</t>
         </is>
@@ -3041,33 +3316,38 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
+          <t>SpecialDevice</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
           <t>SM</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>SM1898</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>CH1 pulse measure start cmd</t>
         </is>
       </c>
-      <c r="E35" t="n">
+      <c r="F35" t="n">
         <v>1</v>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="G35" t="inlineStr">
         <is>
           <t>12ChkPls.csv</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="H35" t="inlineStr">
         <is>
           <t>OUT</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="I35" t="inlineStr">
         <is>
           <t>12ChkPls.csv:row9:step56</t>
         </is>
@@ -3079,33 +3359,38 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
+          <t>SpecialDevice</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
           <t>SM</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>SM1887</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>CH1 error</t>
         </is>
       </c>
-      <c r="E36" t="n">
+      <c r="F36" t="n">
         <v>2</v>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="G36" t="inlineStr">
         <is>
           <t>14RstErr.csv</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="H36" t="inlineStr">
         <is>
           <t>LD</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="I36" t="inlineStr">
         <is>
           <t>14RstErr.csv:row25:step104,14RstErr.csv:row8:step56</t>
         </is>
@@ -3117,33 +3402,38 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
+          <t>SpecialDevice</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
           <t>SM</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>SM1888</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>CH1 warning</t>
         </is>
       </c>
-      <c r="E37" t="n">
+      <c r="F37" t="n">
         <v>2</v>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>14RstErr.csv</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="H37" t="inlineStr">
         <is>
           <t>LD,OR</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="I37" t="inlineStr">
         <is>
           <t>14RstErr.csv:row16:step79,14RstErr.csv:row26:step105</t>
         </is>
@@ -3155,33 +3445,38 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
+          <t>SpecialDevice</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
           <t>SM</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>SM1899</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>CH1 error reset command</t>
         </is>
       </c>
-      <c r="E38" t="n">
+      <c r="F38" t="n">
         <v>1</v>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="G38" t="inlineStr">
         <is>
           <t>14RstErr.csv</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="H38" t="inlineStr">
         <is>
           <t>OUT</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="I38" t="inlineStr">
         <is>
           <t>14RstErr.csv:row28:step107</t>
         </is>
@@ -3193,40 +3488,45 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
+          <t>SpecialDevice</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
           <t>SM</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>SM400</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>Always ON</t>
         </is>
       </c>
-      <c r="E39" t="n">
+      <c r="F39" t="n">
         <v>1</v>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="G39" t="inlineStr">
         <is>
           <t>15Match.csv</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="H39" t="inlineStr">
         <is>
           <t>LD</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>15Match.csv:row16:step69</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H39"/>
+  <autoFilter ref="A1:I39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: add check reference sheet
</commit_message>
<xml_diff>
--- a/output/io_list_report.xlsx
+++ b/output/io_list_report.xlsx
@@ -11,19 +11,21 @@
     <sheet name="INPUT" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="OUTPUT" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="CHECK" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="DEVICE_USAGE" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="INSTRUCTION_REFERENCE" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="DEVICE_TYPE_REFERENCE" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="RAW_DATA" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="CHECK_REFERENCE" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="DEVICE_USAGE" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="INSTRUCTION_REFERENCE" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="DEVICE_TYPE_REFERENCE" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="RAW_DATA" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'INPUT'!$A$1:$I$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'OUTPUT'!$A$1:$I$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CHECK'!$A$1:$F$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'DEVICE_USAGE'!$A$1:$I$39</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'INSTRUCTION_REFERENCE'!$A$1:$D$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'DEVICE_TYPE_REFERENCE'!$A$1:$D$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'RAW_DATA'!$A$1:$F$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'CHECK_REFERENCE'!$A$1:$F$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'DEVICE_USAGE'!$A$1:$I$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'INSTRUCTION_REFERENCE'!$A$1:$D$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'DEVICE_TYPE_REFERENCE'!$A$1:$E$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'RAW_DATA'!$A$1:$F$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -483,7 +485,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-08 14:59:57</t>
+          <t>2026-06-10 14:21:17</t>
         </is>
       </c>
     </row>
@@ -1874,6 +1876,253 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="4" max="4"/>
+    <col width="80" customWidth="1" min="5" max="5"/>
+    <col width="80" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Level</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ReviewPoint</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>SuggestedAction</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>MISSING_DEVICE_COMMENT</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>An X/Y device is used in ladder CSV, but no device comment is registered.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>The signal name or field meaning is unclear from the I/O list.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Check the GX Works2 device comment table or electrical drawing, then add the missing comment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>MISSING_LOGIC_NOTE</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>LogicContext</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>No nearby ladder note was found for the X/Y device.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>This is not always a defect, but the logic context may be harder to understand.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Use DeviceComment as the main source and review the ladder around the listed step if needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>MULTIPLE_USED_FILES</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Usage</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>The same X/Y device is referenced in multiple ladder CSV files.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>A change to this I/O may affect more than one program section.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Open the listed files and confirm whether the shared usage is intentional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>MULTIPLE_LOGIC_NOTES</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>LogicContext</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Multiple ladder notes were linked to the same X/Y device.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>A logic note may describe an operation, not the device name itself.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Compare the notes and use them as context instead of blindly copying them as signal names.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>COMMENTED_BUT_NOT_USED</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>A device comment exists, but the X/Y device was not found in ladder CSV.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>The comment may be obsolete, reserved, or the ladder export may be incomplete.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Confirm whether the address is spare, deleted, or used in a program that was not exported.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SPARE_OR_UNUSED_DEVICE</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>The X/Y device is commented as spare or unused and was not found in ladder CSV.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>This is usually acceptable, but it is useful to keep visible in the report.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Treat as reference information unless the project expects every spare address to be excluded.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F7"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3531,7 +3780,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3794,19 +4043,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="72" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="72" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3817,15 +4067,20 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>UsageCategory</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Meaning</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Example</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
@@ -3839,15 +4094,20 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>PhysicalIO</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>Input</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>X0</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Physical input such as a sensor, push button, or switch.</t>
         </is>
@@ -3861,15 +4121,20 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>PhysicalIO</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>Output</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Y0</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Physical output such as a lamp, relay, solenoid, or actuator signal.</t>
         </is>
@@ -3883,15 +4148,20 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>InternalDevice</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>Internal relay</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>M100</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Internal bit used inside the PLC program.</t>
         </is>
@@ -3900,164 +4170,334 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SM</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Special relay</t>
+          <t>InternalDevice</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SM402</t>
+          <t>Latch relay</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>System bit provided by the PLC CPU or special function area.</t>
+          <t>L100</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Internal bit that can retain its state depending on PLC settings.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Data register</t>
+          <t>InternalDevice</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>D2000</t>
+          <t>Link relay</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Word register used to store numeric values.</t>
+          <t>B10</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Bit device often used for link or network-related data areas.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>W</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Special data register</t>
+          <t>InternalDevice</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>SD1880</t>
+          <t>Link register</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>System data register provided by the PLC CPU or special function area.</t>
+          <t>W10</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Word device often used for link or network-related data areas.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>R</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Decimal constant</t>
+          <t>InternalDevice</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>K1000</t>
+          <t>File register</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Fixed decimal value used as an instruction parameter.</t>
+          <t>R100</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Word register used as an extended data storage area.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>ZR</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Hex constant</t>
+          <t>InternalDevice</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>H1</t>
+          <t>File register</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Fixed hexadecimal value used as an instruction parameter.</t>
+          <t>ZR1000</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Extended file register used as a large data storage area.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>SM</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Timer</t>
+          <t>SpecialDevice</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>T0</t>
+          <t>Special relay</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Timer device used for time-based control.</t>
+          <t>SM402</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>System bit provided by the PLC CPU or special function area.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>InternalDevice</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Data register</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>D2000</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Word register used to store numeric values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>SpecialDevice</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Special data register</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>SD1880</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>System data register provided by the PLC CPU or special function area.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Constant</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Decimal constant</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>K1000</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Fixed decimal value used as an instruction parameter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Constant</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Hex constant</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Fixed hexadecimal value used as an instruction parameter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>TimerCounter</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Timer</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Timer device used for time-based control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>C</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>TimerCounter</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
         <is>
           <t>Counter</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>C0</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>Counter device used for count-based control.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D11"/>
+  <autoFilter ref="A1:E16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
feat: add review workflow columns to check sheet
</commit_message>
<xml_diff>
--- a/output/io_list_report.xlsx
+++ b/output/io_list_report.xlsx
@@ -20,8 +20,8 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'INPUT'!$A$1:$I$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'OUTPUT'!$A$1:$I$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CHECK'!$A$1:$F$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'CHECK_REFERENCE'!$A$1:$F$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CHECK'!$A$1:$I$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'CHECK_REFERENCE'!$A$1:$G$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'DEVICE_USAGE'!$A$1:$I$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'INSTRUCTION_REFERENCE'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'DEVICE_TYPE_REFERENCE'!$A$1:$E$16</definedName>
@@ -485,7 +485,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-10 14:21:17</t>
+          <t>2026-06-11 16:01:14</t>
         </is>
       </c>
     </row>
@@ -1693,15 +1693,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="80" customWidth="1" min="5" max="5"/>
-    <col width="65" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
+    <col width="65" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1712,27 +1715,42 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>ReviewStatus</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Message</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Details</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>ReviewerNote</t>
         </is>
       </c>
     </row>
@@ -1744,29 +1762,40 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
           <t>LogicContext</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>MULTIPLE_LOGIC_NOTES</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>X57</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Multiple logic notes were linked to this device. Review the context before using them as signal descriptions.</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Stores latch cnt val 1 in D2002,Stores latch cnt value in D2002</t>
         </is>
       </c>
+      <c r="I2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1776,29 +1805,40 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
           <t>LogicContext</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>MULTIPLE_LOGIC_NOTES</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>X5C</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Multiple logic notes were linked to this device. Review the context before using them as signal descriptions.</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Coinc sgnl 1 reset cmd:OFF,Coinc sgnl 1 reset cmd:ON</t>
         </is>
       </c>
+      <c r="I3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1808,29 +1848,40 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
           <t>Usage</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>MULTIPLE_USED_FILES</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>X57</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>This I/O device is referenced in multiple ladder CSV files. Check whether the shared usage is intentional.</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>04Lcnt1.csv,08LcPre.csv</t>
         </is>
       </c>
+      <c r="I4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1840,32 +1891,43 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
           <t>LogicContext</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>MISSING_LOGIC_NOTE</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>X61</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>No nearby ladder logic note was found for this device.</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>13OutPwm.csv</t>
         </is>
       </c>
+      <c r="I5" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F5"/>
+  <autoFilter ref="A1:I5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1876,15 +1938,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="80" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
     <col width="80" customWidth="1" min="5" max="5"/>
     <col width="80" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1900,20 +1963,25 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Meaning</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>ReviewPoint</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>SuggestedAction</t>
         </is>
@@ -1932,20 +2000,25 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>Documentation</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>An X/Y device is used in ladder CSV, but no device comment is registered.</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>The signal name or field meaning is unclear from the I/O list.</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Check the GX Works2 device comment table or electrical drawing, then add the missing comment.</t>
         </is>
@@ -1964,20 +2037,25 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>LogicContext</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>No nearby ladder note was found for the X/Y device.</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>This is not always a defect, but the logic context may be harder to understand.</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Use DeviceComment as the main source and review the ladder around the listed step if needed.</t>
         </is>
@@ -1996,20 +2074,25 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>Usage</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>The same X/Y device is referenced in multiple ladder CSV files.</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>A change to this I/O may affect more than one program section.</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Open the listed files and confirm whether the shared usage is intentional.</t>
         </is>
@@ -2028,20 +2111,25 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>LogicContext</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Multiple ladder notes were linked to the same X/Y device.</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>A logic note may describe an operation, not the device name itself.</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Compare the notes and use them as context instead of blindly copying them as signal names.</t>
         </is>
@@ -2060,20 +2148,25 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>Documentation</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>A device comment exists, but the X/Y device was not found in ladder CSV.</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>The comment may be obsolete, reserved, or the ladder export may be incomplete.</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Confirm whether the address is spare, deleted, or used in a program that was not exported.</t>
         </is>
@@ -2092,27 +2185,32 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>Documentation</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>The X/Y device is commented as spare or unused and was not found in ladder CSV.</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>This is usually acceptable, but it is useful to keep visible in the report.</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Treat as reference information unless the project expects every spare address to be excluded.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F7"/>
+  <autoFilter ref="A1:G7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
refactor: optimize report column structure
</commit_message>
<xml_diff>
--- a/output/io_list_report.xlsx
+++ b/output/io_list_report.xlsx
@@ -18,8 +18,8 @@
     <sheet name="RAW_DATA" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'INPUT'!$A$1:$I$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'OUTPUT'!$A$1:$I$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'INPUT'!$A$1:$G$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'OUTPUT'!$A$1:$G$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CHECK'!$A$1:$I$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'CHECK_REFERENCE'!$A$1:$G$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'DEVICE_USAGE'!$A$1:$I$39</definedName>
@@ -485,7 +485,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-13 21:33:31</t>
+          <t>2026-06-17 16:02:08</t>
         </is>
       </c>
     </row>
@@ -648,18 +648,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="65" customWidth="1" min="8" max="8"/>
-    <col width="31" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="31" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="65" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -670,42 +668,32 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Device</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Device</t>
+          <t>DeviceComment</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>DeviceComment</t>
+          <t>UsedFiles</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>AddressNo</t>
+          <t>Steps</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>UsedFiles</t>
+          <t>Instructions</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Instructions</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
           <t>LogicNotes</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Steps</t>
         </is>
       </c>
     </row>
@@ -715,40 +703,32 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>INPUT</t>
+          <t>X50</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>X50</t>
+          <t>CH1 count start signal</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>CH1 count start signal</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>80</v>
+          <t>01CmnPgm.csv</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv:129</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>01CmnPgm.csv</t>
+          <t>LD</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
           <t>Count enable command:ON</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>01CmnPgm.csv:129</t>
         </is>
       </c>
     </row>
@@ -758,40 +738,32 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>INPUT</t>
+          <t>X51</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>X51</t>
+          <t>CH1 count stop signal</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>CH1 count stop signal</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>81</v>
+          <t>01CmnPgm.csv</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv:145</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>01CmnPgm.csv</t>
+          <t>LD</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
           <t>Count enable command:OFF</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>01CmnPgm.csv:145</t>
         </is>
       </c>
     </row>
@@ -801,40 +773,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>INPUT</t>
+          <t>X52</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>X52</t>
+          <t>CH1 current value read signal</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>CH1 current value read signal</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>82</v>
+          <t>01CmnPgm.csv</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>01CmnPgm.csv:161</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>01CmnPgm.csv</t>
+          <t>LD</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
           <t>Stores current value in D2000</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>01CmnPgm.csv:161</t>
         </is>
       </c>
     </row>
@@ -844,40 +808,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>INPUT</t>
+          <t>X53</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>X53</t>
+          <t>CH1 preset command signal</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>CH1 preset command signal</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>83</v>
+          <t>02PreSet.csv</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>02PreSet.csv:52</t>
+        </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>02PreSet.csv</t>
+          <t>LD</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
           <t>Preset command</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>02PreSet.csv:52</t>
         </is>
       </c>
     </row>
@@ -887,40 +843,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>INPUT</t>
+          <t>X54</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>X54</t>
+          <t>CH1 counter fnc exe start signal</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>CH1 counter fnc exe start signal</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>84</v>
+          <t>06DisCnt.csv</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>06DisCnt.csv:55</t>
+        </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>06DisCnt.csv</t>
+          <t>LD</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
           <t>Selected cnt fnc start cmd:ON</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>06DisCnt.csv:55</t>
         </is>
       </c>
     </row>
@@ -930,40 +878,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>INPUT</t>
+          <t>X55</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>X55</t>
+          <t>CH1 counter fnc exe stop signal</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>CH1 counter fnc exe stop signal</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>85</v>
+          <t>06DisCnt.csv</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>06DisCnt.csv:74</t>
+        </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>06DisCnt.csv</t>
+          <t>LD</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
           <t>Selected cnt fnc start cmd:OFF</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>06DisCnt.csv:74</t>
         </is>
       </c>
     </row>
@@ -973,40 +913,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>INPUT</t>
+          <t>X56</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>X56</t>
+          <t>CH1 latch 1 execution cmd signal</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>CH1 latch 1 execution cmd signal</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>86</v>
+          <t>04Lcnt1.csv</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>04Lcnt1.csv:52</t>
+        </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>04Lcnt1.csv</t>
+          <t>LD</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
           <t>Selected counter fnc start cmd</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>04Lcnt1.csv:52</t>
         </is>
       </c>
     </row>
@@ -1016,40 +948,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>INPUT</t>
+          <t>X57</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>X57</t>
+          <t>CH1 latch cnt data 1 read signal</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>CH1 latch cnt data 1 read signal</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>87</v>
+          <t>04Lcnt1.csv,08LcPre.csv</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>04Lcnt1.csv:71,08LcPre.csv:61</t>
+        </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>04Lcnt1.csv,08LcPre.csv</t>
+          <t>LD</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
           <t>Stores latch cnt val 1 in D2002,Stores latch cnt value in D2002</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>04Lcnt1.csv:71,08LcPre.csv:61</t>
         </is>
       </c>
     </row>
@@ -1059,40 +983,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>INPUT</t>
+          <t>X58</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>X58</t>
+          <t>CH1 latch cnt data 2 read signal</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>CH1 latch cnt data 2 read signal</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>88</v>
+          <t>05Lcnt2.csv</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>05Lcnt2.csv:52</t>
+        </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>05Lcnt2.csv</t>
+          <t>LD</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
           <t>Stores latch cnt val 2 in D2004</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>05Lcnt2.csv:52</t>
         </is>
       </c>
     </row>
@@ -1102,40 +1018,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>INPUT</t>
+          <t>X59</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>X59</t>
+          <t>CH1 sampling count start signal</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>CH1 sampling count start signal</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>89</v>
+          <t>07SplCnt.csv</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>07SplCnt.csv:57</t>
+        </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>07SplCnt.csv</t>
+          <t>LD</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
           <t>Selected counter fnc start cmd</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>07SplCnt.csv:57</t>
         </is>
       </c>
     </row>
@@ -1145,40 +1053,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>INPUT</t>
+          <t>X5A</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>X5A</t>
+          <t>CH1 sampling cnt data read signl</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>CH1 sampling cnt data read signl</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>90</v>
+          <t>07SplCnt.csv</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>07SplCnt.csv:76</t>
+        </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>07SplCnt.csv</t>
+          <t>LD</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
           <t>Stores sampling cnt val in D2006</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>07SplCnt.csv:76</t>
         </is>
       </c>
     </row>
@@ -1188,40 +1088,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>INPUT</t>
+          <t>X5B</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>X5B</t>
+          <t>CH1 coinc output enable signal</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>CH1 coinc output enable signal</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>91</v>
+          <t>03MchOut.csv</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>03MchOut.csv:58</t>
+        </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>03MchOut.csv</t>
+          <t>LD</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
           <t>Coincidence output enable cmd</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>03MchOut.csv:58</t>
         </is>
       </c>
     </row>
@@ -1231,40 +1123,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>INPUT</t>
+          <t>X5C</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>X5C</t>
+          <t>CH1 coincidence LED clear signal</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>CH1 coincidence LED clear signal</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>92</v>
+          <t>03MchOut.csv</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>03MchOut.csv:98</t>
+        </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>03MchOut.csv</t>
+          <t>AND</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>AND</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
           <t>Coinc sgnl 1 reset cmd:OFF,Coinc sgnl 1 reset cmd:ON</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>03MchOut.csv:98</t>
         </is>
       </c>
     </row>
@@ -1274,40 +1158,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>INPUT</t>
+          <t>X5D</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>X5D</t>
+          <t>CH1 freq measurement cmd signal</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>CH1 freq measurement cmd signal</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>93</v>
+          <t>10ChkFrq.csv</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>10ChkFrq.csv:57</t>
+        </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>10ChkFrq.csv</t>
+          <t>LD</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
           <t>Stores measured freq in D2008</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>10ChkFrq.csv:57</t>
         </is>
       </c>
     </row>
@@ -1317,40 +1193,32 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>INPUT</t>
+          <t>X5E</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>X5E</t>
+          <t>CH1 rot speed measure cmd signal</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>CH1 rot speed measure cmd signal</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>94</v>
+          <t>11ChkRsp.csv</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>11ChkRsp.csv:58</t>
+        </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>11ChkRsp.csv</t>
+          <t>LD</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
           <t>Stores measured rot spd in D2010</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>11ChkRsp.csv:58</t>
         </is>
       </c>
     </row>
@@ -1360,40 +1228,32 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>INPUT</t>
+          <t>X5F</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>X5F</t>
+          <t>CH1 pulse measurement cmd signal</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>CH1 pulse measurement cmd signal</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>95</v>
+          <t>12ChkPls.csv</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>12ChkPls.csv:55</t>
+        </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>12ChkPls.csv</t>
+          <t>LD</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
           <t>Pulse measurement start command</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>12ChkPls.csv:55</t>
         </is>
       </c>
     </row>
@@ -1403,40 +1263,32 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>INPUT</t>
+          <t>X60</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>X60</t>
+          <t>CH1 measured pulse read signal</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>CH1 measured pulse read signal</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>96</v>
+          <t>12ChkPls.csv</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>12ChkPls.csv:75</t>
+        </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>12ChkPls.csv</t>
+          <t>LD</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
           <t>Stores measured pulse in D2012</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>12ChkPls.csv:75</t>
         </is>
       </c>
     </row>
@@ -1446,38 +1298,30 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>INPUT</t>
+          <t>X61</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>X61</t>
+          <t>CH1 PWM output command signal</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>CH1 PWM output command signal</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>97</v>
+          <t>13OutPwm.csv</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>13OutPwm.csv:86</t>
+        </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>13OutPwm.csv</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
           <t>LD</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>13OutPwm.csv:86</t>
-        </is>
-      </c>
+      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1485,45 +1329,37 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>INPUT</t>
+          <t>X62</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>X62</t>
+          <t>CH1 error reset command signal</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>CH1 error reset command signal</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>98</v>
+          <t>14RstErr.csv</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>14RstErr.csv:103</t>
+        </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>14RstErr.csv</t>
+          <t>LD</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>LD</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
           <t>CH1 error reset command</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>14RstErr.csv:103</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I20"/>
+  <autoFilter ref="A1:G20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1534,18 +1370,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1556,42 +1390,32 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Device</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Device</t>
+          <t>DeviceComment</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>DeviceComment</t>
+          <t>UsedFiles</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>AddressNo</t>
+          <t>Steps</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>UsedFiles</t>
+          <t>Instructions</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Instructions</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
           <t>LogicNotes</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Steps</t>
         </is>
       </c>
     </row>
@@ -1601,40 +1425,32 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>OUTPUT</t>
+          <t>Y70</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Y70</t>
+          <t>CH1 coinc confirmation LED sig</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>CH1 coinc confirmation LED sig</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>112</v>
+          <t>03MchOut.csv</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>03MchOut.csv:80</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>03MchOut.csv</t>
+          <t>OUT</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>OUT</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
           <t>Coincidence conf LED signal</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>03MchOut.csv:80</t>
         </is>
       </c>
     </row>
@@ -1644,45 +1460,37 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>OUTPUT</t>
+          <t>Y71</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Y71</t>
+          <t>CH1 ovrflw occurrence LED signal</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>CH1 ovrflw occurrence LED signal</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>113</v>
+          <t>09ChkOvr.csv</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>09ChkOvr.csv:59</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>09ChkOvr.csv</t>
+          <t>OUT</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>OUT</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
           <t>Overflow confirmation LED signal</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>09ChkOvr.csv:59</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I3"/>
+  <autoFilter ref="A1:G3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1696,7 +1504,7 @@
   <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
@@ -1710,12 +1518,12 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Level</t>
+          <t>Priority</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Priority</t>
+          <t>Severity</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -1730,7 +1538,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>CheckType</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -1745,7 +1553,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Details</t>
+          <t>Evidence</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -1757,12 +1565,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
           <t>WARN</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>P2</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1800,12 +1608,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
           <t>WARN</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>P2</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1843,12 +1651,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
           <t>WARN</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>P2</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1886,12 +1694,12 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
           <t>INFO</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>P3</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -1942,7 +1750,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="80" customWidth="1" min="5" max="5"/>
@@ -1953,12 +1761,12 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>CheckType</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Level</t>
+          <t>Severity</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -2243,7 +2051,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>UsageCategory</t>
+          <t>DeviceCategory</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -2278,7 +2086,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Locations</t>
+          <t>UsageLocations</t>
         </is>
       </c>
     </row>
@@ -4165,7 +3973,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>UsageCategory</t>
+          <t>DeviceCategory</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -4605,8 +4413,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
@@ -4620,12 +4428,12 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>RowNumber</t>
+          <t>CsvRow</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Step</t>
+          <t>StepNo</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">

</xml_diff>